<commit_message>
Modeller güncel verilerle yeniden koşturuldu: N, genç tipleri, ayrışım, tek ödeme eşiği, stok stresi (GUNCEL_MODEL)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gVZQXddJGKmSE7re5wowB
</commit_message>
<xml_diff>
--- a/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
+++ b/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
@@ -612,13 +612,13 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>350000</v>
+        <v>443000</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>700000</v>
+        <v>1966000</v>
       </c>
       <c r="F9" s="4">
         <f>INDEX(C9:E9,$D$2)</f>
@@ -626,7 +626,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Varsayım; veri talebi: GİB, SGK</t>
+          <t>Kötümser: F 3-I 268; İyimser: F 3-I 269 oranları × ILO 2025 (n_veri.py); Orta: geometrik ortalama (Claude)</t>
         </is>
       </c>
     </row>
@@ -5501,10 +5501,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.084463422748595</v>
+        <v>0.7063089484990631</v>
       </c>
       <c r="C4" t="n">
-        <v>2.986259536424468</v>
+        <v>1.839316667074052</v>
       </c>
     </row>
     <row r="5">
@@ -5514,10 +5514,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.863742829232634</v>
+        <v>6.169394495285879</v>
       </c>
       <c r="C5" t="n">
-        <v>14.45167175395206</v>
+        <v>18.41247288760587</v>
       </c>
     </row>
     <row r="6">
@@ -5527,10 +5527,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14.18537328138288</v>
+        <v>39.93106267314105</v>
       </c>
       <c r="C6" t="n">
-        <v>42.73259043346012</v>
+        <v>120.8396531955173</v>
       </c>
     </row>
     <row r="8">
@@ -5547,7 +5547,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4.863742829232634</v>
+        <v>6.169394495285879</v>
       </c>
     </row>
     <row r="10">
@@ -5557,7 +5557,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-1.087615170767367</v>
+        <v>-1.363324344714124</v>
       </c>
     </row>
     <row r="11">
@@ -5567,7 +5567,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3.440481618561076</v>
+        <v>4.367952448635879</v>
       </c>
     </row>
     <row r="12">
@@ -5577,7 +5577,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.823954910190622</v>
+        <v>2.321891500612699</v>
       </c>
     </row>
     <row r="13">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.075453047078635</v>
+        <v>1.374501999588103</v>
       </c>
     </row>
     <row r="14">
@@ -5597,7 +5597,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5.2231600036498</v>
+        <v>6.624313947476747</v>
       </c>
     </row>
     <row r="15">
@@ -5607,7 +5607,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5.490252664609205</v>
+        <v>6.962376944062511</v>
       </c>
     </row>
     <row r="16">
@@ -5617,7 +5617,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4.29473043759288</v>
+        <v>5.449187382438988</v>
       </c>
     </row>
     <row r="17">
@@ -5627,7 +5627,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5.519902244678498</v>
+        <v>6.999904841121647</v>
       </c>
     </row>
     <row r="19">
@@ -5656,7 +5656,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1.371685259209676</v>
+        <v>1.749447342371102</v>
       </c>
     </row>
     <row r="23">
@@ -5666,7 +5666,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1.816043653111378</v>
+        <v>2.311878109509542</v>
       </c>
     </row>
     <row r="24">
@@ -5676,7 +5676,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2.740448089415021</v>
+        <v>3.481910010316724</v>
       </c>
     </row>
     <row r="25">
@@ -5686,7 +5686,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4.210833232420195</v>
+        <v>5.342997491320416</v>
       </c>
     </row>
     <row r="26">
@@ -5696,7 +5696,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>6.348701487779011</v>
+        <v>8.048927883103142</v>
       </c>
     </row>
     <row r="27">
@@ -5706,7 +5706,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>9.050144277377949</v>
+        <v>11.46818261393838</v>
       </c>
     </row>
     <row r="28">
@@ -5716,7 +5716,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>11.31276202009183</v>
+        <v>14.33201021400195</v>
       </c>
     </row>
     <row r="29">
@@ -5743,10 +5743,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>-2.807853045275791</v>
+        <v>-4.815467972647983</v>
       </c>
       <c r="C32" t="n">
-        <v>4.913742829232634</v>
+        <v>21.38180093977515</v>
       </c>
     </row>
     <row r="33">
@@ -5756,10 +5756,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>-1.816846647234291</v>
+        <v>-2.299608756356548</v>
       </c>
       <c r="C33" t="n">
-        <v>2.027565172759112</v>
+        <v>2.566318204377959</v>
       </c>
     </row>
     <row r="34">
@@ -5769,10 +5769,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.8407871839926644</v>
+        <v>1.064196350025002</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.2802623946642227</v>
+        <v>-0.3547321166750012</v>
       </c>
     </row>
     <row r="35">
@@ -5782,10 +5782,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.5857025562826614</v>
+        <v>0.7413320926663408</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.5857025562826629</v>
+        <v>-0.7413320926663408</v>
       </c>
     </row>
     <row r="36">
@@ -5795,10 +5795,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.5589775689572811</v>
+        <v>0.7075058944230738</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.5786323428758425</v>
+        <v>-0.7323832225542812</v>
       </c>
     </row>
     <row r="37">
@@ -5808,10 +5808,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.4880854635688839</v>
+        <v>0.6177767438886175</v>
       </c>
       <c r="C37" t="n">
-        <v>-0.4880854635688858</v>
+        <v>-0.6177767438886175</v>
       </c>
     </row>
     <row r="38">
@@ -5821,10 +5821,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>-0.4620656689140339</v>
+        <v>-0.5848431180826216</v>
       </c>
       <c r="C38" t="n">
-        <v>0.02112601201078796</v>
+        <v>0.02673949520222473</v>
       </c>
     </row>
     <row r="39">
@@ -5834,10 +5834,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.3132549176882858</v>
+        <v>0.3964912243883152</v>
       </c>
       <c r="C39" t="n">
-        <v>-0.3132549176882877</v>
+        <v>-0.3964912243883171</v>
       </c>
     </row>
     <row r="40">
@@ -5847,10 +5847,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.2530813514801616</v>
+        <v>0.3203286820163203</v>
       </c>
       <c r="C40" t="n">
-        <v>-0.2892358302630443</v>
+        <v>-0.3660899223043652</v>
       </c>
     </row>
     <row r="41">
@@ -5860,10 +5860,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.2567265531551189</v>
+        <v>0.3249424658506203</v>
       </c>
       <c r="C41" t="n">
-        <v>-0.2567265531551171</v>
+        <v>-0.3249424658506222</v>
       </c>
     </row>
     <row r="42">
@@ -5873,10 +5873,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.07592440544404792</v>
+        <v>0.0960986046048956</v>
       </c>
       <c r="C42" t="n">
-        <v>-0.1265406757400818</v>
+        <v>-0.1601643410081606</v>
       </c>
     </row>
     <row r="43">
@@ -5886,10 +5886,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.06327033787003994</v>
+        <v>0.08008217050407981</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.1265406757400818</v>
+        <v>-0.1601643410081606</v>
       </c>
     </row>
     <row r="44">
@@ -5899,10 +5899,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>-0.07361091709504318</v>
+        <v>-0.09317038935172653</v>
       </c>
       <c r="C44" t="n">
-        <v>0.07361091709504509</v>
+        <v>0.09317038935172844</v>
       </c>
     </row>
     <row r="45">
@@ -5912,10 +5912,10 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.03464387011085701</v>
+        <v>0.04384924131174183</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.06928774022171402</v>
+        <v>-0.0876984826234827</v>
       </c>
     </row>
     <row r="46">
@@ -5925,10 +5925,10 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>-0.02078632206651497</v>
+        <v>-0.02630954478704452</v>
       </c>
       <c r="C46" t="n">
-        <v>0.02078632206651306</v>
+        <v>0.02630954478704548</v>
       </c>
     </row>
     <row r="47">

</xml_diff>

<commit_message>
F 3-I 273: gayrıresmî tanımı, N güncellemesi, istihdam emsalleri araştırması
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gVZQXddJGKmSE7re5wowB
</commit_message>
<xml_diff>
--- a/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
+++ b/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
@@ -615,10 +615,10 @@
         <v>100000</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>443000</v>
+        <v>331000</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1966000</v>
+        <v>1096000</v>
       </c>
       <c r="F9" s="4">
         <f>INDEX(C9:E9,$D$2)</f>
@@ -626,7 +626,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Kötümser: F 3-I 268; İyimser: F 3-I 269 oranları × ILO 2025 (n_veri.py); Orta: geometrik ortalama (Claude)</t>
+          <t>Kötümser: F 3-I 268; İyimser: F 3-I 269 oranları × ILO 2025 + F 3-I 273 gayrıresmî tanımı (n_veri.py); Orta: geometrik ortalama (Claude)</t>
         </is>
       </c>
     </row>
@@ -5514,10 +5514,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.169394495285879</v>
+        <v>4.596996789931434</v>
       </c>
       <c r="C5" t="n">
-        <v>18.41247288760587</v>
+        <v>13.64247582342064</v>
       </c>
     </row>
     <row r="6">
@@ -5527,10 +5527,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>39.93106267314105</v>
+        <v>22.23852730913662</v>
       </c>
       <c r="C6" t="n">
-        <v>120.8396531955173</v>
+        <v>67.16418352490928</v>
       </c>
     </row>
     <row r="8">
@@ -5547,7 +5547,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6.169394495285879</v>
+        <v>4.596996789931434</v>
       </c>
     </row>
     <row r="10">
@@ -5557,7 +5557,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-1.363324344714124</v>
+        <v>-1.031287490068567</v>
       </c>
     </row>
     <row r="11">
@@ -5567,7 +5567,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.367952448635879</v>
+        <v>3.250998330696333</v>
       </c>
     </row>
     <row r="12">
@@ -5577,7 +5577,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2.321891500612699</v>
+        <v>1.722225929351702</v>
       </c>
     </row>
     <row r="13">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.374501999588103</v>
+        <v>1.014357024522939</v>
       </c>
     </row>
     <row r="14">
@@ -5597,7 +5597,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6.624313947476747</v>
+        <v>4.93690274630881</v>
       </c>
     </row>
     <row r="15">
@@ -5607,7 +5607,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6.962376944062511</v>
+        <v>5.189496091387563</v>
       </c>
     </row>
     <row r="16">
@@ -5617,7 +5617,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5.449187382438988</v>
+        <v>4.058873642409265</v>
       </c>
     </row>
     <row r="17">
@@ -5627,7 +5627,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>6.999904841121647</v>
+        <v>5.217536122824525</v>
       </c>
     </row>
     <row r="19">
@@ -5656,7 +5656,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1.749447342371102</v>
+        <v>1.294508059424006</v>
       </c>
     </row>
     <row r="23">
@@ -5666,7 +5666,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2.311878109509542</v>
+        <v>1.714744140513902</v>
       </c>
     </row>
     <row r="24">
@@ -5676,7 +5676,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.481910010316724</v>
+        <v>2.588966621703916</v>
       </c>
     </row>
     <row r="25">
@@ -5686,7 +5686,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>5.342997491320416</v>
+        <v>3.979530856945953</v>
       </c>
     </row>
     <row r="26">
@@ -5696,7 +5696,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>8.048927883103142</v>
+        <v>6.001343407013863</v>
       </c>
     </row>
     <row r="27">
@@ -5706,7 +5706,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>11.46818261393838</v>
+        <v>8.55613644517743</v>
       </c>
     </row>
     <row r="28">
@@ -5716,7 +5716,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>14.33201021400195</v>
+        <v>10.69592636757256</v>
       </c>
     </row>
     <row r="29">
@@ -5743,10 +5743,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>-4.815467972647983</v>
+        <v>-3.243070267293539</v>
       </c>
       <c r="C32" t="n">
-        <v>21.38180093977515</v>
+        <v>10.7400378981799</v>
       </c>
     </row>
     <row r="33">
@@ -5756,10 +5756,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>-2.299608756356548</v>
+        <v>-1.718217829241573</v>
       </c>
       <c r="C33" t="n">
-        <v>2.566318204377959</v>
+        <v>1.917497349095045</v>
       </c>
     </row>
     <row r="34">
@@ -5769,10 +5769,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1.064196350025002</v>
+        <v>0.7951444511473493</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.3547321166750012</v>
+        <v>-0.2650481503824501</v>
       </c>
     </row>
     <row r="35">
@@ -5782,10 +5782,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.7413320926663408</v>
+        <v>0.5539072746558895</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.7413320926663408</v>
+        <v>-0.5539072746558895</v>
       </c>
     </row>
     <row r="36">
@@ -5795,10 +5795,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.7075058944230738</v>
+        <v>0.5286330723567438</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.7323832225542812</v>
+        <v>-0.5472208728340111</v>
       </c>
     </row>
     <row r="37">
@@ -5808,10 +5808,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.6177767438886175</v>
+        <v>0.4615893955465746</v>
       </c>
       <c r="C37" t="n">
-        <v>-0.6177767438886175</v>
+        <v>-0.4615893955465736</v>
       </c>
     </row>
     <row r="38">
@@ -5821,10 +5821,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>-0.5848431180826216</v>
+        <v>-0.4369821040301309</v>
       </c>
       <c r="C38" t="n">
-        <v>0.02673949520222473</v>
+        <v>0.01997917135877514</v>
       </c>
     </row>
     <row r="39">
@@ -5834,10 +5834,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.3964912243883152</v>
+        <v>0.2962496507280645</v>
       </c>
       <c r="C39" t="n">
-        <v>-0.3964912243883171</v>
+        <v>-0.2962496507280655</v>
       </c>
     </row>
     <row r="40">
@@ -5847,10 +5847,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.3203286820163203</v>
+        <v>0.2393426495426683</v>
       </c>
       <c r="C40" t="n">
-        <v>-0.3660899223043652</v>
+        <v>-0.2735344566201916</v>
       </c>
     </row>
     <row r="41">
@@ -5860,10 +5860,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.3249424658506203</v>
+        <v>0.2427899688409824</v>
       </c>
       <c r="C41" t="n">
-        <v>-0.3249424658506222</v>
+        <v>-0.2427899688409824</v>
       </c>
     </row>
     <row r="42">
@@ -5873,10 +5873,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.0960986046048956</v>
+        <v>0.07180279486279964</v>
       </c>
       <c r="C42" t="n">
-        <v>-0.1601643410081606</v>
+        <v>-0.1196713247713346</v>
       </c>
     </row>
     <row r="43">
@@ -5886,10 +5886,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.08008217050407981</v>
+        <v>0.05983566238566685</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.1601643410081606</v>
+        <v>-0.1196713247713346</v>
       </c>
     </row>
     <row r="44">
@@ -5899,10 +5899,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>-0.09317038935172653</v>
+        <v>-0.06961489588131332</v>
       </c>
       <c r="C44" t="n">
-        <v>0.09317038935172844</v>
+        <v>0.06961489588131332</v>
       </c>
     </row>
     <row r="45">
@@ -5912,10 +5912,10 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.04384924131174183</v>
+        <v>0.03276320287626743</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.0876984826234827</v>
+        <v>-0.06552640575253486</v>
       </c>
     </row>
     <row r="46">
@@ -5925,10 +5925,10 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>-0.02630954478704452</v>
+        <v>-0.01965792172576046</v>
       </c>
       <c r="C46" t="n">
-        <v>0.02630954478704548</v>
+        <v>0.01965792172576046</v>
       </c>
     </row>
     <row r="47">

</xml_diff>

<commit_message>
Mali model: Excel sonuç formülleri kayıtlı prim sürdürme ve (1-s-u) yeni girenle hizalandı; Python çıktı sayfası ve duyarlılık tabloları yenilendi
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gVZQXddJGKmSE7re5wowB
</commit_message>
<xml_diff>
--- a/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
+++ b/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
@@ -5696,11 +5696,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yutulma: prim (TL)</t>
+          <t>Yutulma: eski prim (kayıtlı prim sürer, F 3-I 310: 0)</t>
         </is>
       </c>
       <c r="B11">
-        <f>B5*Girdiler!$F$10*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$M$2:$M$61)</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -5762,11 +5762,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Gelire bağlı yeni prim (TL)</t>
+          <t>Gelire bağlı yeni prim + kayıtlı sürdürülen prim (TL)</t>
         </is>
       </c>
       <c r="B17">
-        <f>B5*(1-Girdiler!$F$15)*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$O$2:$O$61)</f>
+        <f>B5*(1-Girdiler!$F$10-Girdiler!$F$15)*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$O$2:$O$61)+B5*Girdiler!$F$10*Girdiler!$F$28*Girdiler!$F$27</f>
         <v/>
       </c>
     </row>
@@ -5795,7 +5795,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Not: eski sabit prim kalktı; yerine gelire bağlı prim (Girdiler: prim_k, prim_ay); varyantlar Senaryolar_Python sayfasındadır.</t>
+          <t>Not: kayıtlı 4/b primi sürer (F 3-I 310); yeni girenlere gelire bağlı prim; vadeli ceza ve faiz mali modelde yoktur. Varyantlar Senaryolar_Python sayfasındadır.</t>
         </is>
       </c>
     </row>
@@ -5810,7 +5810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -5819,10 +5819,11 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Python modeli çıktıları (statik değerler; model.py ve analiz.py ile üretilir)</t>
-        </is>
-      </c>
-    </row>
+          <t>Python modeli çıktıları (statik değerler; model.py, analiz.py, duyarlilik_tablolari.py ile 17 Oct 2026 üretildi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -5847,10 +5848,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-2.048110252063701</v>
+        <v>4.65</v>
       </c>
       <c r="C4" t="n">
-        <v>-6.518307808347563</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="5">
@@ -5860,10 +5861,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.6413105825489</v>
+        <v>12.66</v>
       </c>
       <c r="C5" t="n">
-        <v>4.674154885402459</v>
+        <v>38.12</v>
       </c>
     </row>
     <row r="6">
@@ -5873,27 +5874,28 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26.56432895445933</v>
+        <v>38.67</v>
       </c>
       <c r="C6" t="n">
-        <v>80.28979116639738</v>
-      </c>
-    </row>
+        <v>117.02</v>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Politika varyantları (Orta, 4. yıl net, mlr TL)</t>
+          <t>Politika varyantları (Orta, 4. yıl net, mlr TL) -- analiz.py</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>V0 Baz: %13,5; gelire bağlı prim, tam prim 6 asgari ücrette</t>
+          <t>V0 Baz: %13,5; gelire bağlı prim, tam prim 6 asgari ücret</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.6413105825489</v>
+        <v>12.66</v>
       </c>
     </row>
     <row r="10">
@@ -5903,7 +5905,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.3955031889298513</v>
+        <v>11.65</v>
       </c>
     </row>
     <row r="11">
@@ -5913,7 +5915,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3.042843900370332</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="12">
@@ -5923,7 +5925,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.000609637259104</v>
+        <v>12.14</v>
       </c>
     </row>
     <row r="13">
@@ -5933,7 +5935,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5.752387877450135</v>
+        <v>16.81</v>
       </c>
     </row>
     <row r="14">
@@ -5943,7 +5945,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>10.19932119480739</v>
+        <v>21.29</v>
       </c>
     </row>
     <row r="15">
@@ -5953,7 +5955,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.875941222046813</v>
+        <v>13.59</v>
       </c>
     </row>
     <row r="16">
@@ -5963,7 +5965,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3.7519171875489</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="17">
@@ -5973,7 +5975,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1.39214910382509</v>
+        <v>12.46</v>
       </c>
     </row>
     <row r="18">
@@ -5983,7 +5985,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-34.75811889395275</v>
+        <v>40.05</v>
       </c>
     </row>
     <row r="19">
@@ -5993,7 +5995,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1.981216538926277</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20">
@@ -6003,23 +6005,27 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2.259064380238804</v>
-      </c>
-    </row>
+        <v>13.28</v>
+      </c>
+    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Kırılma noktası s* (Orta)</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>0.1883279083005191</v>
-      </c>
-    </row>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>yok (analiz.py: None)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Monte Carlo (4000 deneme), 4. yıl net (mlr TL)</t>
+          <t>Monte Carlo (analiz.py), 4. yıl net (mlr TL)</t>
         </is>
       </c>
     </row>
@@ -6030,307 +6036,182 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-16.34800279896533</v>
+        <v>4.73</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-10.95323132106929</v>
+        <v>13.16</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P95</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>-4.96310105473143</v>
+        <v>37.89</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>P50</t>
+          <t>P(net&gt;0)</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>-0.4736696384264011</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>NPV P50</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2.745564477485866</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>P90</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>6.168665916403549</v>
-      </c>
-    </row>
+        <v>39.63</v>
+      </c>
+    </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>P95</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>8.553404119724528</v>
+          <t>Tornado (Orta tabanı, 4. yıl net, düşük / yüksek; analiz.py, 8 parametre)</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>P(net&gt;0)</t>
+          <t>n_toplam</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.4645</v>
+        <v>-8.869999999999999</v>
+      </c>
+      <c r="C32" t="n">
+        <v>29.38</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>duz_oran</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="C33" t="n">
+        <v>8.630000000000001</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Tornado (Orta tabanı, 4. yıl net değişimi, mlr TL)</t>
-        </is>
+          <t>s_kayitli</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>-4.83</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1.61</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>duz_oran</t>
+          <t>prim_odeme</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>-1.88238452487336</v>
+        <v>-2.81</v>
       </c>
       <c r="C35" t="n">
-        <v>8.558010612258492</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>s_kayitli</t>
+          <t>medyan_W</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>6.42342873114735</v>
+        <v>-2.6</v>
       </c>
       <c r="C36" t="n">
-        <v>-2.141142910382449</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>n_toplam</t>
+          <t>prim_k</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>-1.180340618032616</v>
+        <v>1.14</v>
       </c>
       <c r="C37" t="n">
-        <v>3.908920228549581</v>
+        <v>-0.52</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>medyan_W</t>
+          <t>u_ucretli</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>-2.726409764881736</v>
+        <v>0.92</v>
       </c>
       <c r="C38" t="n">
-        <v>2.968999848105354</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>prim_odeme</t>
+          <t>marj</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2.814142140000001</v>
+        <v>0.53</v>
       </c>
       <c r="C39" t="n">
-        <v>-1.407071070000001</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>prim_k</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1.401533317821432</v>
-      </c>
-      <c r="C40" t="n">
-        <v>-0.6407009452897967</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>u_ucretli</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1.234630639497912</v>
-      </c>
-      <c r="C41" t="n">
-        <v>-1.234630639497911</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>prim_toplama</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>-0.6229036968095244</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>sigma</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>-0.6019303148476094</v>
-      </c>
-      <c r="C43" t="n">
-        <v>-0.03328261409559465</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>marj</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>0.5286330723567436</v>
-      </c>
-      <c r="C44" t="n">
-        <v>-0.5472208728340101</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>kdv_donanim_pay</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>0.3088768988449516</v>
-      </c>
-      <c r="C45" t="n">
-        <v>-0.3088768988449516</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>myo_uygun</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>0.2427899688409824</v>
-      </c>
-      <c r="C46" t="n">
-        <v>-0.2427899688409824</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>kgf_alim</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>0.07180279486280036</v>
-      </c>
-      <c r="C47" t="n">
-        <v>-0.1196713247713342</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>kgf_temerrut</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>0.05983566238566685</v>
-      </c>
-      <c r="C48" t="n">
-        <v>-0.1196713247713342</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>bes_vazgecme</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>-0.08308609119838332</v>
-      </c>
-      <c r="C49" t="n">
-        <v>0.08308609119838332</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>phi</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>0.02752440469740677</v>
-      </c>
-      <c r="C50" t="n">
-        <v>-0.05504880939481378</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>onlem</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>-0.01651464281844425</v>
-      </c>
-      <c r="C51" t="n">
-        <v>0.01651464281844401</v>
-      </c>
-    </row>
+        <v>-0.55</v>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mali model: tam 17 parametreli tornado (analiz.py tüm parametreleri yazar), Excel görünüm notu hesaplanan değerden üretilir
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gVZQXddJGKmSE7re5wowB
</commit_message>
<xml_diff>
--- a/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
+++ b/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
@@ -5810,7 +5810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -5819,7 +5819,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Python modeli çıktıları (statik değerler; model.py, analiz.py, duyarlilik_tablolari.py ile 17 Oct 2026 üretildi)</t>
+          <t>Python modeli çıktıları (statik değerler; model.py, analiz.py, duyarlilik_tablolari.py; 17 Oct 2026)</t>
         </is>
       </c>
     </row>
@@ -5884,334 +5884,247 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Politika varyantları (Orta, 4. yıl net, mlr TL) -- analiz.py</t>
+          <t>Tornado (Orta tabanı, 4. yıl net değişimi, mlr TL; analiz.py, 17 parametre, düşük/yüksek uç)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>V0 Baz: %13,5; gelire bağlı prim, tam prim 6 asgari ücret</t>
+          <t>n_toplam</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12.66</v>
+        <v>-8.869999999999999</v>
+      </c>
+      <c r="C9" t="n">
+        <v>29.38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>V1 Gelire bağlı prim hiç alınmasaydı (prim sıfır)</t>
+          <t>duz_oran</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>11.65</v>
+        <v>-1.9</v>
+      </c>
+      <c r="C10" t="n">
+        <v>8.630000000000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>V2 Tam prim eşiği 3 asgari ücret</t>
+          <t>s_kayitli</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13.8</v>
+        <v>-4.83</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1.61</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>V3 Tam prim eşiği 12 asgari ücret</t>
+          <t>prim_odeme</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12.14</v>
+        <v>-2.81</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1.41</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>V4 Oran %20</t>
+          <t>medyan_W</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16.81</v>
+        <v>-2.6</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2.81</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>V6 Oran %27 (üst sınır)</t>
+          <t>prim_k</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>21.29</v>
+        <v>1.14</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-0.52</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>V7 Maaşlı hiç mikro mükellef olmasaydı (u=0)</t>
+          <t>u_ucretli</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>13.59</v>
+        <v>0.92</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-0.92</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>V8 SGK tahsil oranı %50</t>
+          <t>marj</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>10.55</v>
+        <v>0.53</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-0.55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>V9 Gelire bağlı primin tahsil oranı %80</t>
+          <t>sigma</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>12.46</v>
+        <v>-0.54</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-0.05</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>V10 Halen kayıtlıların hepsi geçse (s=%100)</t>
+          <t>prim_toplama</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>40.05</v>
+        <v>-0.51</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>V11 90 gün prim hibesi olmasaydı</t>
+          <t>kdv_donanim_pay</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>13</v>
+        <v>0.31</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-0.31</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>V12 Donanım KDV mahsubu olmasaydı</t>
+          <t>myo_uygun</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>13.28</v>
-      </c>
-    </row>
-    <row r="21"/>
+        <v>0.24</v>
+      </c>
+      <c r="C20" t="n">
+        <v>-0.24</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>kgf_alim</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Kırılma noktası s* (Orta)</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>yok (analiz.py: None)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
+          <t>kgf_temerrut</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>bes_vazgecme</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Monte Carlo (analiz.py), 4. yıl net (mlr TL)</t>
-        </is>
+          <t>phi</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C24" t="n">
+        <v>-0.06</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>onlem</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4.73</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>P50</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>13.16</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>P95</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>37.89</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>P(net&gt;0)</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>NPV P50</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>39.63</v>
-      </c>
-    </row>
+        <v>-0.02</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30"/>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Tornado (Orta tabanı, 4. yıl net, düşük / yüksek; analiz.py, 8 parametre)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>n_toplam</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>-8.869999999999999</v>
-      </c>
-      <c r="C32" t="n">
-        <v>29.38</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>duz_oran</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>-1.9</v>
-      </c>
-      <c r="C33" t="n">
-        <v>8.630000000000001</v>
-      </c>
-    </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>s_kayitli</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>-4.83</v>
-      </c>
-      <c r="C34" t="n">
-        <v>1.61</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>prim_odeme</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>-2.81</v>
-      </c>
-      <c r="C35" t="n">
-        <v>1.41</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>medyan_W</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>-2.6</v>
-      </c>
-      <c r="C36" t="n">
-        <v>2.81</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>prim_k</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="C37" t="n">
-        <v>-0.52</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>u_ucretli</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="C38" t="n">
-        <v>-0.92</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>marj</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="C39" t="n">
-        <v>-0.55</v>
-      </c>
-    </row>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
+      <c r="A34" s="4" t="n"/>
+    </row>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mali model: üç senaryo için tornado (tornado_senaryo.py), çıktılar Excel Senaryolar_Python sayfasına işlendi
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gVZQXddJGKmSE7re5wowB
</commit_message>
<xml_diff>
--- a/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
+++ b/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
@@ -5810,7 +5810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -5823,7 +5823,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -5880,7 +5879,6 @@
         <v>117.02</v>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
@@ -6109,22 +6107,744 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="4" t="n"/>
     </row>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Tornado (Kötümser tabanı, 4. yıl net değişimi, mlr TL; tornado_senaryo.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Parametre</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Düşük uç</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Yüksek uç</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>n_toplam</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" t="n">
+        <v>46.803</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>s_kayitli</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>-2.997</v>
+      </c>
+      <c r="C39" t="n">
+        <v>-0.999</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>duz_oran</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>-0.486</v>
+      </c>
+      <c r="C40" t="n">
+        <v>2.224</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>prim_odeme</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>medyan_W</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>-0.307</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.874</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>u_ucretli</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0.295</v>
+      </c>
+      <c r="C43" t="n">
+        <v>-0.177</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>marj</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="C44" t="n">
+        <v>-0.223</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>prim_k</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="C45" t="n">
+        <v>-0.081</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>sigma</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>-0.157</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.043</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>kdv_donanim_pay</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="C47" t="n">
+        <v>-0.045</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>myo_uygun</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="C48" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>prim_toplama</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>-0.078</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>kgf_alim</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="C50" t="n">
+        <v>-0.018</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>kgf_temerrut</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="C51" t="n">
+        <v>-0.024</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>bes_vazgecme</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>-0.008999999999999999</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.034</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>phi</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C53" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>onlem</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0.014</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Tornado (Orta tabanı, 4. yıl net değişimi, mlr TL; tornado_senaryo.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Parametre</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Düşük uç</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Yüksek uç</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>n_toplam</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>-8.872999999999999</v>
+      </c>
+      <c r="C58" t="n">
+        <v>29.385</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>duz_oran</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>-1.898</v>
+      </c>
+      <c r="C59" t="n">
+        <v>8.625</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>s_kayitli</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>-4.833</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1.611</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>prim_odeme</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>-2.814</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1.407</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>medyan_W</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>-2.603</v>
+      </c>
+      <c r="C62" t="n">
+        <v>2.814</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>prim_k</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1.139</v>
+      </c>
+      <c r="C63" t="n">
+        <v>-0.521</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>u_ucretli</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="C64" t="n">
+        <v>-0.923</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>marj</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>0.529</v>
+      </c>
+      <c r="C65" t="n">
+        <v>-0.547</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>sigma</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>-0.542</v>
+      </c>
+      <c r="C66" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>prim_toplama</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>-0.506</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>kdv_donanim_pay</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>0.309</v>
+      </c>
+      <c r="C68" t="n">
+        <v>-0.309</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>myo_uygun</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="C69" t="n">
+        <v>-0.243</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>kgf_alim</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="C70" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>kgf_temerrut</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C71" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>bes_vazgecme</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>-0.083</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0.083</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>phi</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="C73" t="n">
+        <v>-0.055</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>onlem</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>-0.017</v>
+      </c>
+      <c r="C74" t="n">
+        <v>0.017</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Tornado (İyimser tabanı, 4. yıl net değişimi, mlr TL; tornado_senaryo.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Parametre</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Düşük uç</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Yüksek uç</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>n_toplam</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>-35.186</v>
+      </c>
+      <c r="C78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>duz_oran</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>-7.111</v>
+      </c>
+      <c r="C79" t="n">
+        <v>32.201</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>s_kayitli</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>-5.212</v>
+      </c>
+      <c r="C80" t="n">
+        <v>15.636</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>medyan_W</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>-14.645</v>
+      </c>
+      <c r="C81" t="n">
+        <v>7.07</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>prim_k</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>5.765</v>
+      </c>
+      <c r="C82" t="n">
+        <v>-2.635</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>u_ucretli</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>2.597</v>
+      </c>
+      <c r="C83" t="n">
+        <v>-4.329</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>prim_odeme</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>-3.106</v>
+      </c>
+      <c r="C84" t="n">
+        <v>1.553</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>prim_toplama</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>-2.562</v>
+      </c>
+      <c r="C85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>myo_uygun</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>0.417</v>
+      </c>
+      <c r="C86" t="n">
+        <v>-1.667</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>kdv_donanim_pay</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>0.522</v>
+      </c>
+      <c r="C87" t="n">
+        <v>-1.566</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>sigma</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>-1.121</v>
+      </c>
+      <c r="C88" t="n">
+        <v>-1.222</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>marj</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>1.098</v>
+      </c>
+      <c r="C89" t="n">
+        <v>-1.124</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>bes_vazgecme</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>-0.499</v>
+      </c>
+      <c r="C90" t="n">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>kgf_alim</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="C91" t="n">
+        <v>-0.377</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>kgf_temerrut</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="C92" t="n">
+        <v>-0.377</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>phi</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="C93" t="n">
+        <v>-0.155</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>onlem</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>-0.052</v>
+      </c>
+      <c r="C94" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Müracaat tek metne indirildi; Devlet metninde dinî lafızlar tarafsızlaştırıldı, doğrulanmamış çözüm iddiaları ölçü/kalan risk olarak yeniden yazıldı; genç modeli 2025 nüfusu ile koşuldu; Excel yeniden üretildi
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gVZQXddJGKmSE7re5wowB
</commit_message>
<xml_diff>
--- a/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
+++ b/kanun/MALI_MODEL/MIKRO_MUKELLEF_MALI_MODEL.xlsx
@@ -543,22 +543,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Medyan yıllık hasılat (asgari ücret katı)</t>
+          <t>Ortalama yıllık hasılat (asgari ücret katı; veri: girişim ciro/firma, 2024)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>medyan_W</t>
+          <t>ort_H_W</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="F7" s="4">
         <f>INDEX(C7:E7,$D$2)</f>
@@ -566,7 +566,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Veri: 2024 genç/mikro ciro ortalaması (ciro/firma, veri_kalibrasyon.json)</t>
         </is>
       </c>
     </row>
@@ -582,13 +582,13 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.9</v>
+        <v>2</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9</v>
+        <v>1.75</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="F8" s="4">
         <f>INDEX(C8:E8,$D$2)</f>
@@ -596,7 +596,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Varsayım: 1,25–2,0 aralığı; veriyle belirlenmez</t>
         </is>
       </c>
     </row>
@@ -612,13 +612,13 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>100000</v>
+        <v>119000</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>331000</v>
+        <v>238000</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1096000</v>
+        <v>475000</v>
       </c>
       <c r="F9" s="4">
         <f>INDEX(C9:E9,$D$2)</f>
@@ -1926,7 +1926,7 @@
         <v/>
       </c>
       <c r="E2">
-        <f>(NORMSDIST((LN(C2)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B2)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C2)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B2)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F2">
@@ -1987,7 +1987,7 @@
         <v/>
       </c>
       <c r="E3">
-        <f>(NORMSDIST((LN(C3)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B3)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C3)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B3)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F3">
@@ -2048,7 +2048,7 @@
         <v/>
       </c>
       <c r="E4">
-        <f>(NORMSDIST((LN(C4)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B4)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C4)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B4)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F4">
@@ -2109,7 +2109,7 @@
         <v/>
       </c>
       <c r="E5">
-        <f>(NORMSDIST((LN(C5)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B5)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C5)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B5)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F5">
@@ -2170,7 +2170,7 @@
         <v/>
       </c>
       <c r="E6">
-        <f>(NORMSDIST((LN(C6)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B6)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C6)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B6)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F6">
@@ -2231,7 +2231,7 @@
         <v/>
       </c>
       <c r="E7">
-        <f>(NORMSDIST((LN(C7)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B7)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C7)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B7)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F7">
@@ -2292,7 +2292,7 @@
         <v/>
       </c>
       <c r="E8">
-        <f>(NORMSDIST((LN(C8)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B8)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C8)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B8)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F8">
@@ -2353,7 +2353,7 @@
         <v/>
       </c>
       <c r="E9">
-        <f>(NORMSDIST((LN(C9)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B9)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C9)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B9)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F9">
@@ -2414,7 +2414,7 @@
         <v/>
       </c>
       <c r="E10">
-        <f>(NORMSDIST((LN(C10)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B10)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C10)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B10)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F10">
@@ -2475,7 +2475,7 @@
         <v/>
       </c>
       <c r="E11">
-        <f>(NORMSDIST((LN(C11)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B11)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C11)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B11)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F11">
@@ -2536,7 +2536,7 @@
         <v/>
       </c>
       <c r="E12">
-        <f>(NORMSDIST((LN(C12)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B12)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C12)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B12)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F12">
@@ -2597,7 +2597,7 @@
         <v/>
       </c>
       <c r="E13">
-        <f>(NORMSDIST((LN(C13)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B13)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C13)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B13)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F13">
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="E14">
-        <f>(NORMSDIST((LN(C14)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B14)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C14)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B14)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F14">
@@ -2719,7 +2719,7 @@
         <v/>
       </c>
       <c r="E15">
-        <f>(NORMSDIST((LN(C15)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B15)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C15)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B15)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F15">
@@ -2780,7 +2780,7 @@
         <v/>
       </c>
       <c r="E16">
-        <f>(NORMSDIST((LN(C16)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B16)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C16)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B16)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F16">
@@ -2841,7 +2841,7 @@
         <v/>
       </c>
       <c r="E17">
-        <f>(NORMSDIST((LN(C17)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B17)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C17)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B17)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F17">
@@ -2902,7 +2902,7 @@
         <v/>
       </c>
       <c r="E18">
-        <f>(NORMSDIST((LN(C18)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B18)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C18)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B18)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F18">
@@ -2963,7 +2963,7 @@
         <v/>
       </c>
       <c r="E19">
-        <f>(NORMSDIST((LN(C19)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B19)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C19)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B19)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F19">
@@ -3024,7 +3024,7 @@
         <v/>
       </c>
       <c r="E20">
-        <f>(NORMSDIST((LN(C20)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B20)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C20)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B20)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F20">
@@ -3085,7 +3085,7 @@
         <v/>
       </c>
       <c r="E21">
-        <f>(NORMSDIST((LN(C21)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B21)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C21)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B21)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F21">
@@ -3146,7 +3146,7 @@
         <v/>
       </c>
       <c r="E22">
-        <f>(NORMSDIST((LN(C22)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B22)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C22)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B22)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F22">
@@ -3207,7 +3207,7 @@
         <v/>
       </c>
       <c r="E23">
-        <f>(NORMSDIST((LN(C23)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B23)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C23)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B23)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F23">
@@ -3268,7 +3268,7 @@
         <v/>
       </c>
       <c r="E24">
-        <f>(NORMSDIST((LN(C24)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B24)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C24)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B24)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F24">
@@ -3329,7 +3329,7 @@
         <v/>
       </c>
       <c r="E25">
-        <f>(NORMSDIST((LN(C25)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B25)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C25)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B25)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F25">
@@ -3390,7 +3390,7 @@
         <v/>
       </c>
       <c r="E26">
-        <f>(NORMSDIST((LN(C26)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B26)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C26)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B26)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F26">
@@ -3451,7 +3451,7 @@
         <v/>
       </c>
       <c r="E27">
-        <f>(NORMSDIST((LN(C27)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B27)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C27)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B27)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F27">
@@ -3512,7 +3512,7 @@
         <v/>
       </c>
       <c r="E28">
-        <f>(NORMSDIST((LN(C28)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B28)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C28)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B28)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F28">
@@ -3573,7 +3573,7 @@
         <v/>
       </c>
       <c r="E29">
-        <f>(NORMSDIST((LN(C29)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B29)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C29)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B29)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F29">
@@ -3634,7 +3634,7 @@
         <v/>
       </c>
       <c r="E30">
-        <f>(NORMSDIST((LN(C30)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B30)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C30)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B30)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F30">
@@ -3695,7 +3695,7 @@
         <v/>
       </c>
       <c r="E31">
-        <f>(NORMSDIST((LN(C31)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B31)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C31)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B31)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F31">
@@ -3756,7 +3756,7 @@
         <v/>
       </c>
       <c r="E32">
-        <f>(NORMSDIST((LN(C32)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B32)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C32)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B32)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F32">
@@ -3817,7 +3817,7 @@
         <v/>
       </c>
       <c r="E33">
-        <f>(NORMSDIST((LN(C33)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B33)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C33)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B33)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F33">
@@ -3878,7 +3878,7 @@
         <v/>
       </c>
       <c r="E34">
-        <f>(NORMSDIST((LN(C34)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B34)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C34)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B34)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F34">
@@ -3939,7 +3939,7 @@
         <v/>
       </c>
       <c r="E35">
-        <f>(NORMSDIST((LN(C35)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B35)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C35)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B35)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F35">
@@ -4000,7 +4000,7 @@
         <v/>
       </c>
       <c r="E36">
-        <f>(NORMSDIST((LN(C36)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B36)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C36)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B36)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F36">
@@ -4061,7 +4061,7 @@
         <v/>
       </c>
       <c r="E37">
-        <f>(NORMSDIST((LN(C37)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B37)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C37)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B37)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F37">
@@ -4122,7 +4122,7 @@
         <v/>
       </c>
       <c r="E38">
-        <f>(NORMSDIST((LN(C38)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B38)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C38)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B38)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F38">
@@ -4183,7 +4183,7 @@
         <v/>
       </c>
       <c r="E39">
-        <f>(NORMSDIST((LN(C39)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B39)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C39)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B39)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F39">
@@ -4244,7 +4244,7 @@
         <v/>
       </c>
       <c r="E40">
-        <f>(NORMSDIST((LN(C40)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B40)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C40)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B40)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F40">
@@ -4305,7 +4305,7 @@
         <v/>
       </c>
       <c r="E41">
-        <f>(NORMSDIST((LN(C41)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B41)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C41)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B41)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F41">
@@ -4366,7 +4366,7 @@
         <v/>
       </c>
       <c r="E42">
-        <f>(NORMSDIST((LN(C42)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B42)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C42)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B42)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F42">
@@ -4427,7 +4427,7 @@
         <v/>
       </c>
       <c r="E43">
-        <f>(NORMSDIST((LN(C43)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B43)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C43)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B43)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F43">
@@ -4488,7 +4488,7 @@
         <v/>
       </c>
       <c r="E44">
-        <f>(NORMSDIST((LN(C44)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B44)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C44)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B44)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F44">
@@ -4549,7 +4549,7 @@
         <v/>
       </c>
       <c r="E45">
-        <f>(NORMSDIST((LN(C45)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B45)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C45)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B45)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F45">
@@ -4610,7 +4610,7 @@
         <v/>
       </c>
       <c r="E46">
-        <f>(NORMSDIST((LN(C46)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B46)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C46)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B46)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F46">
@@ -4671,7 +4671,7 @@
         <v/>
       </c>
       <c r="E47">
-        <f>(NORMSDIST((LN(C47)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B47)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C47)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B47)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F47">
@@ -4732,7 +4732,7 @@
         <v/>
       </c>
       <c r="E48">
-        <f>(NORMSDIST((LN(C48)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B48)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C48)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B48)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F48">
@@ -4793,7 +4793,7 @@
         <v/>
       </c>
       <c r="E49">
-        <f>(NORMSDIST((LN(C49)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B49)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C49)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B49)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F49">
@@ -4854,7 +4854,7 @@
         <v/>
       </c>
       <c r="E50">
-        <f>(NORMSDIST((LN(C50)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B50)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C50)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B50)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F50">
@@ -4915,7 +4915,7 @@
         <v/>
       </c>
       <c r="E51">
-        <f>(NORMSDIST((LN(C51)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B51)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C51)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B51)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F51">
@@ -4976,7 +4976,7 @@
         <v/>
       </c>
       <c r="E52">
-        <f>(NORMSDIST((LN(C52)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B52)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C52)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B52)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F52">
@@ -5037,7 +5037,7 @@
         <v/>
       </c>
       <c r="E53">
-        <f>(NORMSDIST((LN(C53)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B53)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C53)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B53)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F53">
@@ -5098,7 +5098,7 @@
         <v/>
       </c>
       <c r="E54">
-        <f>(NORMSDIST((LN(C54)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B54)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C54)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B54)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F54">
@@ -5159,7 +5159,7 @@
         <v/>
       </c>
       <c r="E55">
-        <f>(NORMSDIST((LN(C55)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B55)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C55)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B55)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F55">
@@ -5220,7 +5220,7 @@
         <v/>
       </c>
       <c r="E56">
-        <f>(NORMSDIST((LN(C56)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B56)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C56)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B56)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F56">
@@ -5281,7 +5281,7 @@
         <v/>
       </c>
       <c r="E57">
-        <f>(NORMSDIST((LN(C57)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B57)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C57)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B57)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F57">
@@ -5342,7 +5342,7 @@
         <v/>
       </c>
       <c r="E58">
-        <f>(NORMSDIST((LN(C58)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B58)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C58)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B58)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F58">
@@ -5403,7 +5403,7 @@
         <v/>
       </c>
       <c r="E59">
-        <f>(NORMSDIST((LN(C59)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B59)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C59)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B59)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F59">
@@ -5464,7 +5464,7 @@
         <v/>
       </c>
       <c r="E60">
-        <f>(NORMSDIST((LN(C60)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B60)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C60)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B60)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F60">
@@ -5525,7 +5525,7 @@
         <v/>
       </c>
       <c r="E61">
-        <f>(NORMSDIST((LN(C61)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN(B61)-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6))/Girdiler!$F$8))</f>
+        <f>(NORMSDIST((LN(C61)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN(B61)-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))/(NORMSDIST((LN((24*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8)-NORMSDIST((LN((0.1*Girdiler!$F$6))-LN(Girdiler!$F$7*Girdiler!$F$6)-Girdiler!$F$8^2/2)/Girdiler!$F$8))</f>
         <v/>
       </c>
       <c r="F61">
@@ -5696,11 +5696,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yutulma: eski prim (kayıtlı prim sürer, F 3-I 310: 0)</t>
+          <t>Yutulma: prim (TL)</t>
         </is>
       </c>
       <c r="B11">
-        <f>0</f>
+        <f>B5*Girdiler!$F$10*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$M$2:$M$61)</f>
         <v/>
       </c>
     </row>
@@ -5762,11 +5762,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Gelire bağlı yeni prim + kayıtlı sürdürülen prim (TL)</t>
+          <t>Gelire bağlı yeni prim (TL)</t>
         </is>
       </c>
       <c r="B17">
-        <f>B5*(1-Girdiler!$F$10-Girdiler!$F$15)*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$O$2:$O$61)+B5*Girdiler!$F$10*Girdiler!$F$28*Girdiler!$F$27</f>
+        <f>B5*(1-Girdiler!$F$15)*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$O$2:$O$61)</f>
         <v/>
       </c>
     </row>
@@ -5795,7 +5795,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Not: kayıtlı 4/b primi sürer (F 3-I 310); yeni girenlere gelire bağlı prim; vadeli ceza ve faiz mali modelde yoktur. Varyantlar Senaryolar_Python sayfasındadır.</t>
+          <t>Not: eski sabit prim kalktı; yerine gelire bağlı prim (Girdiler: prim_k, prim_ay); varyantlar Senaryolar_Python sayfasındadır.</t>
         </is>
       </c>
     </row>
@@ -5810,7 +5810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -5819,7 +5819,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Python modeli çıktıları (statik değerler; model.py, analiz.py, duyarlilik_tablolari.py; 17 Oct 2026)</t>
+          <t>Python modeli çıktıları (statik değerler; model.py ve analiz.py ile üretilir)</t>
         </is>
       </c>
     </row>
@@ -5847,10 +5847,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4.65</v>
+        <v>2.362713726652236</v>
       </c>
       <c r="C4" t="n">
-        <v>13.8</v>
+        <v>6.865098760648426</v>
       </c>
     </row>
     <row r="5">
@@ -5860,10 +5860,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12.66</v>
+        <v>3.778491091574925</v>
       </c>
       <c r="C5" t="n">
-        <v>38.12</v>
+        <v>11.15980229717435</v>
       </c>
     </row>
     <row r="6">
@@ -5873,976 +5873,464 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>38.67</v>
+        <v>11.03746021660951</v>
       </c>
       <c r="C6" t="n">
-        <v>117.02</v>
+        <v>33.18314605534334</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Tornado (Orta tabanı, 4. yıl net değişimi, mlr TL; analiz.py, 17 parametre, düşük/yüksek uç)</t>
+          <t>Politika varyantları (Orta, 4. yıl net, mlr TL)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>n_toplam</t>
+          <t>V0 Baz: %13,5; gelire bağlı prim, tam prim 6 asgari ücrette</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-8.869999999999999</v>
-      </c>
-      <c r="C9" t="n">
-        <v>29.38</v>
+        <v>3.778491091574925</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>duz_oran</t>
+          <t>V1 Gelire bağlı prim hiç alınmasaydı (prim sıfır)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-1.9</v>
-      </c>
-      <c r="C10" t="n">
-        <v>8.630000000000001</v>
+        <v>3.297369139916137</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>s_kayitli</t>
+          <t>V2 Tam prim eşiği 3 asgari ücret</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-4.83</v>
-      </c>
-      <c r="C11" t="n">
-        <v>1.61</v>
+        <v>4.319753287191062</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>prim_odeme</t>
+          <t>V3 Tam prim eşiği 12 asgari ücret</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-2.81</v>
-      </c>
-      <c r="C12" t="n">
-        <v>1.41</v>
+        <v>3.531056945007549</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>medyan_W</t>
+          <t>V4 Oran %20</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-2.6</v>
-      </c>
-      <c r="C13" t="n">
-        <v>2.81</v>
+        <v>7.143855407463859</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>prim_k</t>
+          <t>V6 Oran %27 (üst sınır)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="C14" t="n">
-        <v>-0.52</v>
+        <v>10.77707457633699</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>u_ucretli</t>
+          <t>V7 Maaşlı hiç mikro mükellef olmasaydı (u=0)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="C15" t="n">
-        <v>-0.92</v>
+        <v>4.516714898277905</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>marj</t>
+          <t>V8 SGK tahsil oranı %50</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="C16" t="n">
-        <v>-0.55</v>
+        <v>3.778491091574925</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>V9 Gelire bağlı primin tahsil oranı %80</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.54</v>
-      </c>
-      <c r="C17" t="n">
-        <v>-0.05</v>
+        <v>3.682266701243167</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>prim_toplama</t>
+          <t>V10 Halen kayıtlıların hepsi geçse (s=%100)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.51</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0</v>
+        <v>1.562205462325526</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>kdv_donanim_pay</t>
+          <t>V11 90 gün prim hibesi olmasaydı</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="C19" t="n">
-        <v>-0.31</v>
+        <v>4.165578998564803</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>myo_uygun</t>
+          <t>V12 Donanım KDV mahsubu olmasaydı</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="C20" t="n">
-        <v>-0.24</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>kgf_alim</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="C21" t="n">
-        <v>-0.12</v>
+        <v>4.183867624784411</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>kgf_temerrut</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="C22" t="n">
-        <v>-0.12</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>bes_vazgecme</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>-0.08</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.08</v>
+          <t>Kırılma noktası s* (Orta)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>yok</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>phi</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="C24" t="n">
-        <v>-0.06</v>
+          <t>Monte Carlo (4000 deneme), 4. yıl net (mlr TL)</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>onlem</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.02</v>
+        <v>1.721298851608765</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2.171931583986423</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>P25</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3.165843159128112</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>4.834027296098787</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>P75</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>7.245703013255524</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>10.33375607192481</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>P95</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>12.64466616835029</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>P(net&gt;0)</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n"/>
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Tornado (Orta tabanı, 4. yıl net değişimi, mlr TL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>duz_oran</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>-1.545409391219779</v>
+      </c>
+      <c r="C35" t="n">
+        <v>6.998583484762066</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Tornado (Kötümser tabanı, 4. yıl net değişimi, mlr TL; tornado_senaryo.py)</t>
-        </is>
+          <t>n_toplam</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>-1.914245545787463</v>
+      </c>
+      <c r="C36" t="n">
+        <v>3.8124049945515</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Parametre</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Düşük uç</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Yüksek uç</t>
-        </is>
+          <t>s_kayitli</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2.120868244037097</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1.253437469379797</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>n_toplam</t>
+          <t>sigma</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0</v>
+        <v>2.057404232673791</v>
       </c>
       <c r="C38" t="n">
-        <v>46.803</v>
+        <v>-0.7174174347846322</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>s_kayitli</t>
+          <t>marj</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>-2.997</v>
+        <v>0.9123060500407854</v>
       </c>
       <c r="C39" t="n">
-        <v>-0.999</v>
+        <v>-0.9782161612364202</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>duz_oran</t>
+          <t>ort_H_W</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>-0.486</v>
+        <v>-0.4353148267566376</v>
       </c>
       <c r="C40" t="n">
-        <v>2.224</v>
+        <v>0.8165253356944194</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>prim_odeme</t>
+          <t>u_ucretli</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>-1.7</v>
+        <v>0.7382238067029796</v>
       </c>
       <c r="C41" t="n">
-        <v>0.85</v>
+        <v>-0.7382238067029796</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>medyan_W</t>
+          <t>prim_k</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>-0.307</v>
+        <v>0.541262195616137</v>
       </c>
       <c r="C42" t="n">
-        <v>0.874</v>
+        <v>-0.2474341465673761</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>u_ucretli</t>
+          <t>myo_uygun</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.295</v>
+        <v>0.2764913621356277</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.177</v>
+        <v>-0.2764913621356277</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>marj</t>
+          <t>prim_toplama</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.215</v>
+        <v>-0.2405609758293934</v>
       </c>
       <c r="C44" t="n">
-        <v>-0.223</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>prim_k</t>
+          <t>kdv_donanim_pay</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.176</v>
+        <v>0.202688266604743</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.081</v>
+        <v>-0.202688266604743</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>kgf_alim</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>-0.157</v>
+        <v>0.05741740718800926</v>
       </c>
       <c r="C46" t="n">
-        <v>0.043</v>
+        <v>-0.09569567864668274</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>kdv_donanim_pay</t>
+          <t>kgf_temerrut</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.135</v>
+        <v>0.04784783932334089</v>
       </c>
       <c r="C47" t="n">
-        <v>-0.045</v>
+        <v>-0.09569567864668274</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>myo_uygun</t>
+          <t>bes_vazgecme</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.082</v>
+        <v>-0.06644014260326767</v>
       </c>
       <c r="C48" t="n">
-        <v>-0.02</v>
+        <v>0.06644014260326862</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>prim_toplama</t>
+          <t>phi</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>-0.078</v>
+        <v>0.02201000608873701</v>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>-0.04402001217747402</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>kgf_alim</t>
+          <t>onlem</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.055</v>
+        <v>-0.01320600365324211</v>
       </c>
       <c r="C50" t="n">
-        <v>-0.018</v>
+        <v>0.01320600365324211</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>kgf_temerrut</t>
+          <t>prim_odeme</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.049</v>
+        <v>0</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.024</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>bes_vazgecme</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>-0.008999999999999999</v>
-      </c>
-      <c r="C52" t="n">
-        <v>0.034</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>phi</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="C53" t="n">
-        <v>-0.01</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>onlem</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>-0.003</v>
-      </c>
-      <c r="C54" t="n">
-        <v>0.014</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Tornado (Orta tabanı, 4. yıl net değişimi, mlr TL; tornado_senaryo.py)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Parametre</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Düşük uç</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Yüksek uç</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>n_toplam</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>-8.872999999999999</v>
-      </c>
-      <c r="C58" t="n">
-        <v>29.385</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>duz_oran</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>-1.898</v>
-      </c>
-      <c r="C59" t="n">
-        <v>8.625</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>s_kayitli</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>-4.833</v>
-      </c>
-      <c r="C60" t="n">
-        <v>1.611</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>prim_odeme</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>-2.814</v>
-      </c>
-      <c r="C61" t="n">
-        <v>1.407</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>medyan_W</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>-2.603</v>
-      </c>
-      <c r="C62" t="n">
-        <v>2.814</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>prim_k</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>1.139</v>
-      </c>
-      <c r="C63" t="n">
-        <v>-0.521</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>u_ucretli</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>0.923</v>
-      </c>
-      <c r="C64" t="n">
-        <v>-0.923</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>marj</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>0.529</v>
-      </c>
-      <c r="C65" t="n">
-        <v>-0.547</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>sigma</t>
-        </is>
-      </c>
-      <c r="B66" t="n">
-        <v>-0.542</v>
-      </c>
-      <c r="C66" t="n">
-        <v>-0.05</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>prim_toplama</t>
-        </is>
-      </c>
-      <c r="B67" t="n">
-        <v>-0.506</v>
-      </c>
-      <c r="C67" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>kdv_donanim_pay</t>
-        </is>
-      </c>
-      <c r="B68" t="n">
-        <v>0.309</v>
-      </c>
-      <c r="C68" t="n">
-        <v>-0.309</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>myo_uygun</t>
-        </is>
-      </c>
-      <c r="B69" t="n">
-        <v>0.243</v>
-      </c>
-      <c r="C69" t="n">
-        <v>-0.243</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>kgf_alim</t>
-        </is>
-      </c>
-      <c r="B70" t="n">
-        <v>0.07199999999999999</v>
-      </c>
-      <c r="C70" t="n">
-        <v>-0.12</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>kgf_temerrut</t>
-        </is>
-      </c>
-      <c r="B71" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="C71" t="n">
-        <v>-0.12</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>bes_vazgecme</t>
-        </is>
-      </c>
-      <c r="B72" t="n">
-        <v>-0.083</v>
-      </c>
-      <c r="C72" t="n">
-        <v>0.083</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>phi</t>
-        </is>
-      </c>
-      <c r="B73" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="C73" t="n">
-        <v>-0.055</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>onlem</t>
-        </is>
-      </c>
-      <c r="B74" t="n">
-        <v>-0.017</v>
-      </c>
-      <c r="C74" t="n">
-        <v>0.017</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Tornado (İyimser tabanı, 4. yıl net değişimi, mlr TL; tornado_senaryo.py)</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Parametre</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Düşük uç</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Yüksek uç</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>n_toplam</t>
-        </is>
-      </c>
-      <c r="B78" t="n">
-        <v>-35.186</v>
-      </c>
-      <c r="C78" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>duz_oran</t>
-        </is>
-      </c>
-      <c r="B79" t="n">
-        <v>-7.111</v>
-      </c>
-      <c r="C79" t="n">
-        <v>32.201</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>s_kayitli</t>
-        </is>
-      </c>
-      <c r="B80" t="n">
-        <v>-5.212</v>
-      </c>
-      <c r="C80" t="n">
-        <v>15.636</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>medyan_W</t>
-        </is>
-      </c>
-      <c r="B81" t="n">
-        <v>-14.645</v>
-      </c>
-      <c r="C81" t="n">
-        <v>7.07</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>prim_k</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>5.765</v>
-      </c>
-      <c r="C82" t="n">
-        <v>-2.635</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>u_ucretli</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>2.597</v>
-      </c>
-      <c r="C83" t="n">
-        <v>-4.329</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>prim_odeme</t>
-        </is>
-      </c>
-      <c r="B84" t="n">
-        <v>-3.106</v>
-      </c>
-      <c r="C84" t="n">
-        <v>1.553</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>prim_toplama</t>
-        </is>
-      </c>
-      <c r="B85" t="n">
-        <v>-2.562</v>
-      </c>
-      <c r="C85" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>myo_uygun</t>
-        </is>
-      </c>
-      <c r="B86" t="n">
-        <v>0.417</v>
-      </c>
-      <c r="C86" t="n">
-        <v>-1.667</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>kdv_donanim_pay</t>
-        </is>
-      </c>
-      <c r="B87" t="n">
-        <v>0.522</v>
-      </c>
-      <c r="C87" t="n">
-        <v>-1.566</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>sigma</t>
-        </is>
-      </c>
-      <c r="B88" t="n">
-        <v>-1.121</v>
-      </c>
-      <c r="C88" t="n">
-        <v>-1.222</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>marj</t>
-        </is>
-      </c>
-      <c r="B89" t="n">
-        <v>1.098</v>
-      </c>
-      <c r="C89" t="n">
-        <v>-1.124</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>bes_vazgecme</t>
-        </is>
-      </c>
-      <c r="B90" t="n">
-        <v>-0.499</v>
-      </c>
-      <c r="C90" t="n">
-        <v>0.125</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>kgf_alim</t>
-        </is>
-      </c>
-      <c r="B91" t="n">
-        <v>0.054</v>
-      </c>
-      <c r="C91" t="n">
-        <v>-0.377</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>kgf_temerrut</t>
-        </is>
-      </c>
-      <c r="B92" t="n">
-        <v>0.027</v>
-      </c>
-      <c r="C92" t="n">
-        <v>-0.377</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>phi</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="C93" t="n">
-        <v>-0.155</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>onlem</t>
-        </is>
-      </c>
-      <c r="B94" t="n">
-        <v>-0.052</v>
-      </c>
-      <c r="C94" t="n">
-        <v>0.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>